<commit_message>
Add labour to the kit cost calculator at 10 min per kit
At ten minutes a kit valued at twenty dollars an hour, labour is $3.33
per kit, around seven percent of the $45.99 price. It has never been
counted in any margin figure before. Marked amber as provisional, since
the hourly rate is a placeholder for whatever Maya decides her time is
worth.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dXMz3yKWzn5zTjQb1w6uz
</commit_message>
<xml_diff>
--- a/finance/cogs/kit-cost-calculator.xlsx
+++ b/finance/cogs/kit-cost-calculator.xlsx
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -695,13 +695,17 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="2" t="inlineStr"/>
+          <t>Your labour (10 min/kit)</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>10 min/kit CONFIRMED by Maya, valued at $20/hr. Change the rate to what your time is worth.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -983,6 +987,13 @@
       <c r="A44" s="20" t="inlineStr">
         <is>
           <t>AMBER cells are real but PROVISIONAL - a trial price or a placeholder. Treat as a ceiling, replace with a production quote.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>Labour was never counted before 2026-09-19. At 10 min/kit it is ~7% of the $45.99 price.</t>
         </is>
       </c>
     </row>

</xml_diff>